<commit_message>
chore(weekly-sync): auto-pull through 2026-07-05
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week27.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week27.xlsx
@@ -10898,10 +10898,10 @@
         <v>7584</v>
       </c>
       <c r="G374" t="n">
-        <v>1770.34</v>
+        <v>3540.68</v>
       </c>
       <c r="H374" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="375">

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-07-06
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week27.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week27.xlsx
@@ -1798,10 +1798,10 @@
         <v>5618</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>2965.25</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -2610,10 +2610,10 @@
         <v>11860</v>
       </c>
       <c r="G78" t="n">
-        <v>20240.67</v>
+        <v>20641.52</v>
       </c>
       <c r="H78" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79">
@@ -4010,10 +4010,10 @@
         <v>104103</v>
       </c>
       <c r="G128" t="n">
-        <v>0</v>
+        <v>1324.58</v>
       </c>
       <c r="H128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -5914,10 +5914,10 @@
         <v>31426</v>
       </c>
       <c r="G196" t="n">
-        <v>23609.33</v>
+        <v>25744.08</v>
       </c>
       <c r="H196" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="197">
@@ -9834,10 +9834,10 @@
         <v>21698</v>
       </c>
       <c r="G336" t="n">
-        <v>0</v>
+        <v>2244.92</v>
       </c>
       <c r="H336" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="337">

</xml_diff>